<commit_message>
Done working almost everything
</commit_message>
<xml_diff>
--- a/equation.xlsx
+++ b/equation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\solar-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B8F63CC-6D3A-4F58-8593-8D049DDCE9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00395615-9FCD-432E-B9E3-202F5F5DF2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8A332098-1D51-4CFA-BC61-E45DF4692AB2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
   <si>
     <t>Name</t>
   </si>
@@ -36,9 +36,6 @@
     <t>End</t>
   </si>
   <si>
-    <t>Percentage</t>
-  </si>
-  <si>
     <t>Mercury</t>
   </si>
   <si>
@@ -70,6 +67,12 @@
   </si>
   <si>
     <t>Neptune</t>
+  </si>
+  <si>
+    <t>Percentage [680vh]</t>
+  </si>
+  <si>
+    <t>Percentage [980vh]</t>
   </si>
 </sst>
 </file>
@@ -101,7 +104,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -110,6 +113,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -193,11 +205,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -209,28 +243,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -547,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9687B3B-F3C3-4EAC-BF63-418EECE802F6}">
-  <dimension ref="B1:F17"/>
+  <dimension ref="B1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="21.33203125" customWidth="1"/>
@@ -559,28 +603,28 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="11">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="9">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="D3" s="4">
         <v>20</v>
@@ -588,17 +632,17 @@
       <c r="E3" s="4">
         <v>80</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="12">
         <f>(((E3)-20)/620*100)</f>
         <v>9.67741935483871</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="9">
+      <c r="B4" s="11">
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="4">
         <f>E3</f>
@@ -608,17 +652,17 @@
         <f>D4+60</f>
         <v>140</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="12">
         <f t="shared" ref="F4:F12" si="0">(((E4)-20)/620*100)</f>
         <v>19.35483870967742</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="9">
+      <c r="B5" s="11">
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4">
         <f t="shared" ref="D5:D12" si="1">E4</f>
@@ -628,17 +672,17 @@
         <f t="shared" ref="E5:E12" si="2">D5+60</f>
         <v>200</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="12">
         <f t="shared" si="0"/>
         <v>29.032258064516132</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="9">
+      <c r="B6" s="11">
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4">
         <f t="shared" si="1"/>
@@ -648,17 +692,17 @@
         <f t="shared" si="2"/>
         <v>260</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="12">
         <f t="shared" si="0"/>
         <v>38.70967741935484</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="9">
+      <c r="B7" s="11">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" s="4">
         <f t="shared" si="1"/>
@@ -668,17 +712,17 @@
         <f t="shared" si="2"/>
         <v>320</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="12">
         <f t="shared" si="0"/>
         <v>48.387096774193552</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="9">
+      <c r="B8" s="11">
         <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="4">
         <f t="shared" si="1"/>
@@ -688,17 +732,17 @@
         <f t="shared" si="2"/>
         <v>380</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="12">
         <f t="shared" si="0"/>
         <v>58.064516129032263</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="9">
+      <c r="B9" s="11">
         <v>7</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="4">
         <f t="shared" si="1"/>
@@ -708,17 +752,17 @@
         <f t="shared" si="2"/>
         <v>440</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="12">
         <f t="shared" si="0"/>
         <v>67.741935483870961</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="4">
         <f t="shared" si="1"/>
@@ -728,17 +772,17 @@
         <f t="shared" si="2"/>
         <v>500</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="12">
         <f t="shared" si="0"/>
         <v>77.41935483870968</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="9">
+      <c r="B11" s="11">
         <v>9</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="4">
         <f t="shared" si="1"/>
@@ -748,27 +792,27 @@
         <f t="shared" si="2"/>
         <v>560</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="12">
         <f t="shared" si="0"/>
         <v>87.096774193548384</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="11">
+      <c r="B12" s="13">
         <v>10</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="13">
+      <c r="C12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="15">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="15">
         <f t="shared" si="2"/>
         <v>620</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="16">
         <f t="shared" si="0"/>
         <v>96.774193548387103</v>
       </c>
@@ -779,19 +823,224 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="B15" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F17" s="1"/>
+      <c r="B16" s="11">
+        <v>1</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="4">
+        <v>20</v>
+      </c>
+      <c r="E16" s="4">
+        <v>80</v>
+      </c>
+      <c r="F16" s="12">
+        <f>(((E16)-20)/980*100)</f>
+        <v>6.1224489795918364</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="11">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="4">
+        <f>E16</f>
+        <v>80</v>
+      </c>
+      <c r="E17" s="4">
+        <f>D17+100</f>
+        <v>180</v>
+      </c>
+      <c r="F17" s="12">
+        <f>(((E17)-20)/980*100)</f>
+        <v>16.326530612244898</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="11">
+        <v>3</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" s="4">
+        <f t="shared" ref="D18:D25" si="3">E17</f>
+        <v>180</v>
+      </c>
+      <c r="E18" s="4">
+        <f t="shared" ref="E18:E25" si="4">D18+100</f>
+        <v>280</v>
+      </c>
+      <c r="F18" s="12">
+        <f t="shared" ref="F18:F25" si="5">(((E18)-20)/980*100)</f>
+        <v>26.530612244897959</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="11">
+        <v>4</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="4">
+        <f t="shared" si="3"/>
+        <v>280</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" si="4"/>
+        <v>380</v>
+      </c>
+      <c r="F19" s="12">
+        <f t="shared" si="5"/>
+        <v>36.734693877551024</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="11">
+        <v>5</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="4">
+        <f t="shared" si="3"/>
+        <v>380</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" si="4"/>
+        <v>480</v>
+      </c>
+      <c r="F20" s="12">
+        <f t="shared" si="5"/>
+        <v>46.938775510204081</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="11">
+        <v>6</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="4">
+        <f t="shared" si="3"/>
+        <v>480</v>
+      </c>
+      <c r="E21" s="4">
+        <f t="shared" si="4"/>
+        <v>580</v>
+      </c>
+      <c r="F21" s="12">
+        <f t="shared" si="5"/>
+        <v>57.142857142857139</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="11">
+        <v>7</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="4">
+        <f t="shared" si="3"/>
+        <v>580</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" si="4"/>
+        <v>680</v>
+      </c>
+      <c r="F22" s="12">
+        <f t="shared" si="5"/>
+        <v>67.346938775510196</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="11">
+        <v>8</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="4">
+        <f t="shared" si="3"/>
+        <v>680</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" si="4"/>
+        <v>780</v>
+      </c>
+      <c r="F23" s="12">
+        <f t="shared" si="5"/>
+        <v>77.551020408163268</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="11">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="4">
+        <f t="shared" si="3"/>
+        <v>780</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="4"/>
+        <v>880</v>
+      </c>
+      <c r="F24" s="12">
+        <f t="shared" si="5"/>
+        <v>87.755102040816325</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="17">
+        <v>10</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="6">
+        <f t="shared" si="3"/>
+        <v>880</v>
+      </c>
+      <c r="E25" s="6">
+        <f t="shared" si="4"/>
+        <v>980</v>
+      </c>
+      <c r="F25" s="18">
+        <f t="shared" si="5"/>
+        <v>97.959183673469383</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>